<commit_message>
Table 2 shows Models 1-4 (Model 2 = adiposity + HbA1c + CRP); supplementary tables consolidated to S1-S5 (annotation merged into S1)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/publication_package/03_Tables/Main_Tables.xlsx
+++ b/publication_package/03_Tables/Main_Tables.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="250">
   <si>
     <t>Characteristic</t>
   </si>
@@ -596,24 +596,39 @@
     <t>1.06 (1.04–1.08)</t>
   </si>
   <si>
+    <t>Model 2</t>
+  </si>
+  <si>
+    <t>1.03 (1.01–1.05)</t>
+  </si>
+  <si>
+    <t>1.00 (0.98–1.02)</t>
+  </si>
+  <si>
+    <t>1.02 (1.00–1.04)</t>
+  </si>
+  <si>
+    <t>0.97 (0.95–0.99)</t>
+  </si>
+  <si>
+    <t>1.06 (1.03–1.08)</t>
+  </si>
+  <si>
+    <t>0.98 (0.96–0.99)</t>
+  </si>
+  <si>
+    <t>0.93 (0.91–0.95)</t>
+  </si>
+  <si>
     <t>Model 3</t>
   </si>
   <si>
-    <t>1.00 (0.98–1.02)</t>
-  </si>
-  <si>
-    <t>1.02 (1.00–1.04)</t>
-  </si>
-  <si>
     <t>1.00 (0.98–1.01)</t>
   </si>
   <si>
     <t>1.07 (1.05–1.09)</t>
   </si>
   <si>
-    <t>0.98 (0.96–0.99)</t>
-  </si>
-  <si>
     <t>0.92 (0.90–0.94)</t>
   </si>
   <si>
@@ -626,18 +641,12 @@
     <t>1.04 (1.02–1.06)</t>
   </si>
   <si>
-    <t>1.03 (1.01–1.05)</t>
-  </si>
-  <si>
     <t>0.99 (0.98–1.01)</t>
   </si>
   <si>
     <t>0.98 (0.97–1.00)</t>
   </si>
   <si>
-    <t>0.93 (0.91–0.95)</t>
-  </si>
-  <si>
     <t>0.94 (0.92–0.96)</t>
   </si>
   <si>
@@ -677,6 +686,36 @@
     <t>1.03 (1.00–1.05)</t>
   </si>
   <si>
+    <t>1.07 (1.04–1.10)</t>
+  </si>
+  <si>
+    <t>0.87 (0.84–0.90)</t>
+  </si>
+  <si>
+    <t>0.90 (0.88–0.93)</t>
+  </si>
+  <si>
+    <t>0.95 (0.93–0.97)</t>
+  </si>
+  <si>
+    <t>0.97 (0.95–1.00)</t>
+  </si>
+  <si>
+    <t>0.92 (0.90–0.95)</t>
+  </si>
+  <si>
+    <t>1.12 (1.09–1.16)</t>
+  </si>
+  <si>
+    <t>0.93 (0.90–0.95)</t>
+  </si>
+  <si>
+    <t>1.11 (1.08–1.15)</t>
+  </si>
+  <si>
+    <t>1.02 (0.99–1.04)</t>
+  </si>
+  <si>
     <t>1.09 (1.06–1.12)</t>
   </si>
   <si>
@@ -695,9 +734,6 @@
     <t>1.07 (1.05–1.10)</t>
   </si>
   <si>
-    <t>0.93 (0.90–0.95)</t>
-  </si>
-  <si>
     <t>1.11 (1.08–1.14)</t>
   </si>
   <si>
@@ -708,9 +744,6 @@
   </si>
   <si>
     <t>0.90 (0.87–0.93)</t>
-  </si>
-  <si>
-    <t>0.92 (0.90–0.95)</t>
   </si>
   <si>
     <t>0.99 (0.97–1.02)</t>
@@ -1883,10 +1916,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>162</v>
       </c>
@@ -1895,13 +1928,15 @@
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="1"/>
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" spans="1:9">
       <c r="B2" t="s">
         <v>179</v>
       </c>
@@ -1912,21 +1947,27 @@
         <v>199</v>
       </c>
       <c r="E2" t="s">
+        <v>204</v>
+      </c>
+      <c r="F2" t="s">
         <v>179</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>191</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="I2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>164</v>
       </c>
@@ -1934,22 +1975,28 @@
         <v>180</v>
       </c>
       <c r="C4" t="s">
+        <v>192</v>
+      </c>
+      <c r="D4" t="s">
         <v>180</v>
       </c>
-      <c r="D4" t="s">
-        <v>200</v>
-      </c>
       <c r="E4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F4" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="G4" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+        <v>221</v>
+      </c>
+      <c r="H4" t="s">
+        <v>231</v>
+      </c>
+      <c r="I4" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>165</v>
       </c>
@@ -1957,22 +2004,28 @@
         <v>181</v>
       </c>
       <c r="C5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D5" t="s">
         <v>193</v>
       </c>
       <c r="E5" t="s">
-        <v>207</v>
+        <v>194</v>
       </c>
       <c r="F5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G5" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+        <v>222</v>
+      </c>
+      <c r="H5" t="s">
+        <v>211</v>
+      </c>
+      <c r="I5" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>166</v>
       </c>
@@ -1980,22 +2033,28 @@
         <v>182</v>
       </c>
       <c r="C6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D6" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="E6" t="s">
-        <v>208</v>
+        <v>192</v>
       </c>
       <c r="F6" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="G6" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>223</v>
+      </c>
+      <c r="H6" t="s">
+        <v>232</v>
+      </c>
+      <c r="I6" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>167</v>
       </c>
@@ -2003,22 +2062,28 @@
         <v>183</v>
       </c>
       <c r="C7" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D7" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E7" t="s">
-        <v>209</v>
+        <v>193</v>
       </c>
       <c r="F7" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="G7" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+        <v>224</v>
+      </c>
+      <c r="H7" t="s">
+        <v>233</v>
+      </c>
+      <c r="I7" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
         <v>168</v>
       </c>
@@ -2026,22 +2091,28 @@
         <v>183</v>
       </c>
       <c r="C8" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="D8" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E8" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="F8" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="G8" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+        <v>225</v>
+      </c>
+      <c r="H8" t="s">
+        <v>234</v>
+      </c>
+      <c r="I8" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
         <v>169</v>
       </c>
@@ -2049,22 +2120,28 @@
         <v>184</v>
       </c>
       <c r="C9" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D9" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E9" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="F9" t="s">
-        <v>222</v>
+        <v>202</v>
       </c>
       <c r="G9" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+        <v>226</v>
+      </c>
+      <c r="H9" t="s">
+        <v>235</v>
+      </c>
+      <c r="I9" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
         <v>170</v>
       </c>
@@ -2072,27 +2149,33 @@
         <v>185</v>
       </c>
       <c r="C10" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="D10" t="s">
+        <v>201</v>
+      </c>
+      <c r="E10" t="s">
         <v>180</v>
       </c>
-      <c r="E10" t="s">
-        <v>211</v>
-      </c>
       <c r="F10" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="G10" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+        <v>209</v>
+      </c>
+      <c r="H10" t="s">
+        <v>236</v>
+      </c>
+      <c r="I10" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
         <v>172</v>
       </c>
@@ -2100,22 +2183,28 @@
         <v>186</v>
       </c>
       <c r="C12" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D12" t="s">
+        <v>201</v>
+      </c>
+      <c r="E12" t="s">
         <v>180</v>
       </c>
-      <c r="E12" t="s">
-        <v>212</v>
-      </c>
       <c r="F12" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="G12" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+        <v>227</v>
+      </c>
+      <c r="H12" t="s">
+        <v>214</v>
+      </c>
+      <c r="I12" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
         <v>173</v>
       </c>
@@ -2123,27 +2212,33 @@
         <v>183</v>
       </c>
       <c r="C13" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D13" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="E13" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="F13" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="G13" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+        <v>212</v>
+      </c>
+      <c r="H13" t="s">
+        <v>212</v>
+      </c>
+      <c r="I13" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
       <c r="A14" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:9">
       <c r="A15" t="s">
         <v>175</v>
       </c>
@@ -2151,22 +2246,28 @@
         <v>187</v>
       </c>
       <c r="C15" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="D15" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="E15" t="s">
-        <v>214</v>
+        <v>198</v>
       </c>
       <c r="F15" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="G15" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
+        <v>226</v>
+      </c>
+      <c r="H15" t="s">
+        <v>216</v>
+      </c>
+      <c r="I15" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
       <c r="A16" t="s">
         <v>176</v>
       </c>
@@ -2177,19 +2278,25 @@
         <v>198</v>
       </c>
       <c r="D16" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="E16" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="F16" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="G16" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
+        <v>228</v>
+      </c>
+      <c r="H16" t="s">
+        <v>228</v>
+      </c>
+      <c r="I16" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>177</v>
       </c>
@@ -2197,22 +2304,28 @@
         <v>189</v>
       </c>
       <c r="C17" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="D17" t="s">
+        <v>201</v>
+      </c>
+      <c r="E17" t="s">
         <v>180</v>
       </c>
-      <c r="E17" t="s">
-        <v>216</v>
-      </c>
       <c r="F17" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="G17" t="s">
+        <v>229</v>
+      </c>
+      <c r="H17" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="18" spans="1:7">
+      <c r="I17" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>178</v>
       </c>
@@ -2220,19 +2333,25 @@
         <v>190</v>
       </c>
       <c r="C18" t="s">
+        <v>180</v>
+      </c>
+      <c r="D18" t="s">
         <v>190</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>180</v>
       </c>
-      <c r="E18" t="s">
-        <v>217</v>
-      </c>
       <c r="F18" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="G18" t="s">
+        <v>230</v>
+      </c>
+      <c r="H18" t="s">
         <v>238</v>
+      </c>
+      <c r="I18" t="s">
+        <v>249</v>
       </c>
     </row>
   </sheetData>

</xml_diff>